<commit_message>
Harden live runs: retry policy, transient-error caching, blocked sites, http fallback, DNS and Excel edge cases
- Never honour Retry-After for page fetches; return the final status instead of RetryError
- Do not cache Overpass runtime errors or VIES busy answers; VIES retries bypass the cache
- robots.txt / bot challenges / rate limits are 'blocked' (unverified), not 'dead'
- Retry scheme-less websites over http when https fails
- Compare e-mails case-insensitively; SERVFAIL is 'unknown', not 'undeliverable'
- Excel: strip control characters, keep '=' text as text, write CSV/JSON first, fall back when the workbook is locked
- Ctrl+C cancels queued fetches; CLI/dashboard show source warnings on failure; YAML dates accepted
- Regression tests for each case
</commit_message>
<xml_diff>
--- a/data/output/samples/kortrijk_restaurants_sample.xlsx
+++ b/data/output/samples/kortrijk_restaurants_sample.xlsx
@@ -1247,7 +1247,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-08 08:53</t>
+          <t>2026-09-08 09:30</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       <c r="AG2" s="11" t="n"/>
       <c r="AH2" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI2" s="11" t="n"/>
@@ -1782,7 +1782,7 @@
       <c r="AG3" s="11" t="n"/>
       <c r="AH3" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI3" s="11" t="n"/>
@@ -1922,7 +1922,7 @@
       <c r="AG4" s="11" t="n"/>
       <c r="AH4" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI4" s="11" t="n"/>
@@ -2046,7 +2046,7 @@
       <c r="AG5" s="11" t="n"/>
       <c r="AH5" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI5" s="11" t="n"/>
@@ -2186,7 +2186,7 @@
       <c r="AG6" s="11" t="n"/>
       <c r="AH6" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI6" s="11" t="n"/>
@@ -2302,7 +2302,7 @@
       <c r="AG7" s="11" t="n"/>
       <c r="AH7" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI7" s="11" t="n"/>
@@ -2418,7 +2418,7 @@
       <c r="AG8" s="11" t="n"/>
       <c r="AH8" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI8" s="11" t="n"/>
@@ -2530,7 +2530,7 @@
       <c r="AG9" s="11" t="n"/>
       <c r="AH9" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI9" s="11" t="n"/>
@@ -2654,7 +2654,7 @@
       <c r="AG10" s="11" t="n"/>
       <c r="AH10" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI10" s="11" t="n"/>
@@ -2786,7 +2786,7 @@
       <c r="AG11" s="11" t="n"/>
       <c r="AH11" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI11" s="11" t="n"/>
@@ -2902,7 +2902,7 @@
       <c r="AG12" s="11" t="n"/>
       <c r="AH12" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI12" s="11" t="n"/>
@@ -3018,7 +3018,7 @@
       <c r="AG13" s="11" t="n"/>
       <c r="AH13" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI13" s="11" t="n"/>
@@ -3146,7 +3146,7 @@
       <c r="AG14" s="11" t="n"/>
       <c r="AH14" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI14" s="11" t="n"/>
@@ -3254,7 +3254,7 @@
       <c r="AG15" s="11" t="n"/>
       <c r="AH15" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI15" s="11" t="n"/>
@@ -3386,7 +3386,7 @@
       <c r="AG16" s="11" t="n"/>
       <c r="AH16" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI16" s="11" t="n"/>
@@ -3486,7 +3486,7 @@
       <c r="AG17" s="11" t="n"/>
       <c r="AH17" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI17" s="11" t="n"/>
@@ -3586,7 +3586,7 @@
       <c r="AG18" s="11" t="n"/>
       <c r="AH18" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI18" s="11" t="n"/>
@@ -3702,7 +3702,7 @@
       <c r="AG19" s="11" t="n"/>
       <c r="AH19" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI19" s="11" t="n"/>
@@ -3802,7 +3802,7 @@
       <c r="AG20" s="11" t="n"/>
       <c r="AH20" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI20" s="11" t="n"/>
@@ -3918,7 +3918,7 @@
       <c r="AG21" s="11" t="n"/>
       <c r="AH21" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI21" s="11" t="n"/>
@@ -4050,7 +4050,7 @@
       <c r="AG22" s="11" t="n"/>
       <c r="AH22" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI22" s="11" t="n"/>
@@ -4166,7 +4166,7 @@
       <c r="AG23" s="11" t="n"/>
       <c r="AH23" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI23" s="11" t="n"/>
@@ -4282,7 +4282,7 @@
       <c r="AG24" s="11" t="n"/>
       <c r="AH24" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI24" s="11" t="n"/>
@@ -4398,7 +4398,7 @@
       <c r="AG25" s="11" t="n"/>
       <c r="AH25" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI25" s="11" t="n"/>
@@ -4526,7 +4526,7 @@
       <c r="AG26" s="11" t="n"/>
       <c r="AH26" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI26" s="11" t="n"/>
@@ -4654,7 +4654,7 @@
       <c r="AG27" s="11" t="n"/>
       <c r="AH27" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI27" s="11" t="n"/>
@@ -4778,7 +4778,7 @@
       <c r="AG28" s="11" t="n"/>
       <c r="AH28" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI28" s="11" t="n"/>
@@ -4878,7 +4878,7 @@
       <c r="AG29" s="11" t="n"/>
       <c r="AH29" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI29" s="11" t="n"/>
@@ -5010,7 +5010,7 @@
       <c r="AG30" s="11" t="n"/>
       <c r="AH30" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI30" s="11" t="n"/>
@@ -5138,7 +5138,7 @@
       <c r="AG31" s="11" t="n"/>
       <c r="AH31" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI31" s="11" t="n"/>
@@ -5242,7 +5242,7 @@
       <c r="AG32" s="11" t="n"/>
       <c r="AH32" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI32" s="11" t="n"/>
@@ -5366,7 +5366,7 @@
       <c r="AG33" s="11" t="n"/>
       <c r="AH33" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI33" s="11" t="n"/>
@@ -5494,7 +5494,7 @@
       <c r="AG34" s="11" t="n"/>
       <c r="AH34" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI34" s="11" t="n"/>
@@ -5622,7 +5622,7 @@
       <c r="AG35" s="11" t="n"/>
       <c r="AH35" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI35" s="11" t="n"/>
@@ -5730,7 +5730,7 @@
       <c r="AG36" s="11" t="n"/>
       <c r="AH36" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI36" s="11" t="n"/>
@@ -5850,7 +5850,7 @@
       <c r="AG37" s="11" t="n"/>
       <c r="AH37" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI37" s="11" t="n"/>
@@ -5970,7 +5970,7 @@
       <c r="AG38" s="11" t="n"/>
       <c r="AH38" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI38" s="11" t="n"/>
@@ -6094,7 +6094,7 @@
       <c r="AG39" s="11" t="n"/>
       <c r="AH39" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI39" s="11" t="n"/>
@@ -6214,7 +6214,7 @@
       <c r="AG40" s="11" t="n"/>
       <c r="AH40" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI40" s="11" t="n"/>
@@ -6326,7 +6326,7 @@
       <c r="AG41" s="11" t="n"/>
       <c r="AH41" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI41" s="11" t="n"/>
@@ -6434,7 +6434,7 @@
       <c r="AG42" s="11" t="n"/>
       <c r="AH42" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI42" s="11" t="n"/>
@@ -6566,7 +6566,7 @@
       <c r="AG43" s="11" t="n"/>
       <c r="AH43" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI43" s="11" t="n"/>
@@ -6670,7 +6670,7 @@
       <c r="AG44" s="11" t="n"/>
       <c r="AH44" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI44" s="11" t="n"/>
@@ -6790,7 +6790,7 @@
       <c r="AG45" s="11" t="n"/>
       <c r="AH45" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI45" s="11" t="n"/>
@@ -6926,7 +6926,7 @@
       <c r="AG46" s="11" t="n"/>
       <c r="AH46" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI46" s="11" t="n"/>
@@ -7050,7 +7050,7 @@
       <c r="AG47" s="11" t="n"/>
       <c r="AH47" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI47" s="11" t="n"/>
@@ -7182,7 +7182,7 @@
       <c r="AG48" s="11" t="n"/>
       <c r="AH48" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI48" s="11" t="n"/>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="AH49" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI49" s="11" t="n"/>
@@ -7436,7 +7436,7 @@
       </c>
       <c r="AH50" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI50" s="11" t="n"/>
@@ -7582,7 +7582,7 @@
       </c>
       <c r="AH51" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI51" s="11" t="n"/>
@@ -7699,7 +7699,7 @@
       </c>
       <c r="AH52" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI52" s="11" t="n"/>
@@ -7835,7 +7835,7 @@
       <c r="AG53" s="11" t="n"/>
       <c r="AH53" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI53" s="11" t="n"/>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="AH54" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI54" s="11" t="n"/>
@@ -8084,7 +8084,7 @@
       <c r="AG55" s="11" t="n"/>
       <c r="AH55" s="11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
       <c r="AI55" s="11" t="n"/>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-08T08:53:56+00:00</t>
+          <t>2026-09-08T09:30:49+00:00</t>
         </is>
       </c>
     </row>
@@ -9552,7 +9552,7 @@
         <v>60</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>

</xml_diff>